<commit_message>
Keep BOH internal accounting independent of MISA
</commit_message>
<xml_diff>
--- a/public/templates/BOH-task.xlsx
+++ b/public/templates/BOH-task.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entry" sheetId="1" r:id="R81e843064e7e45fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="Rfafe92a83e144036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entry" sheetId="1" r:id="R9d215931666948e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R6427041cb9b14a3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1335,7 +1335,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="E2:E101">
-      <x:formula1>"Payroll,Bank,Student invoices,Tax filing,Contracts,Admin,Work log"</x:formula1>
+      <x:formula1>"Payroll,Bank,Student invoices,Contracts,Admin,Work log"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G2:G101">
       <x:formula1>"To do,In progress,Done,Logged in source"</x:formula1>
@@ -1343,7 +1343,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac7c84e6aa1e4e06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raebb94286100471f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1524,7 +1524,7 @@
         <x:v>No / Không</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>Payroll, Bank, Student invoices, Tax filing, Contracts, Admin, Work log</x:v>
+        <x:v>Payroll, Bank, Student invoices, Contracts, Admin, Work log</x:v>
       </x:c>
       <x:c r="E16" s="5" t="str">
         <x:v>Payroll</x:v>

</xml_diff>